<commit_message>
Fix HTML report plots: show datapoints, add regression equation and R2
</commit_message>
<xml_diff>
--- a/Water_2H_Report.xlsx
+++ b/Water_2H_Report.xlsx
@@ -1238,10 +1238,10 @@
         <v>-94.89</v>
       </c>
       <c r="C2" t="n">
-        <v>-93.15807747429326</v>
+        <v>-93.15807747429319</v>
       </c>
       <c r="D2" t="n">
-        <v>1.731922525706736</v>
+        <v>1.731922525706807</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>
@@ -1381,7 +1381,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1.248369180421077</v>
+        <v>1.248369180421079</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
Fix invisible plots: disable binary encoding and use explicit lists for Plotly data
</commit_message>
<xml_diff>
--- a/Water_2H_Report.xlsx
+++ b/Water_2H_Report.xlsx
@@ -1238,10 +1238,10 @@
         <v>-94.89</v>
       </c>
       <c r="C2" t="n">
-        <v>-93.15807747429319</v>
+        <v>-93.15807747429325</v>
       </c>
       <c r="D2" t="n">
-        <v>1.731922525706807</v>
+        <v>1.73192252570675</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>
@@ -1381,7 +1381,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1.248369180421079</v>
+        <v>1.248369180421078</v>
       </c>
     </row>
     <row r="12">

</xml_diff>